<commit_message>
Add authorized vendors Excel file
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PRUEBASEXTRACTOR\Automatizacion\WhatsApp\botvendedores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BDDB5B-31BD-43D3-8479-135E0DFF7812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD145D1-42D0-4C6A-976A-BA1E95E28B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>ABDEL MARTIN ARGOTT CARRASCO</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>JEFE DE VENTAS</t>
-  </si>
-  <si>
-    <t>SUPERVISOR ARCOR</t>
   </si>
 </sst>
 </file>
@@ -404,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE86CED-79C6-4198-8C8C-911AFBD57A57}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.109375" bestFit="1" customWidth="1"/>
@@ -566,17 +563,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>940246472</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Actualización: WEBHOOK_VENDEDORES_V2 (períodos dinámicos, días laborables reales) 📋 vendedores.xlsx incluido en repo
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PRUEBASEXTRACTOR\Automatizacion\WhatsApp\botvendedores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD145D1-42D0-4C6A-976A-BA1E95E28B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4F88256-DF1C-42A4-877F-26FCBAACCC0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="16">
   <si>
     <t>ABDEL MARTIN ARGOTT CARRASCO</t>
   </si>
@@ -62,6 +62,12 @@
   </si>
   <si>
     <t>JEFE DE VENTAS</t>
+  </si>
+  <si>
+    <t>VENDEDOR</t>
+  </si>
+  <si>
+    <t>ADMINISTRADOR</t>
   </si>
 </sst>
 </file>
@@ -401,15 +407,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE86CED-79C6-4198-8C8C-911AFBD57A57}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -419,8 +426,11 @@
       <c r="C1">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -430,8 +440,11 @@
       <c r="C2">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -441,8 +454,11 @@
       <c r="C3">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -452,8 +468,11 @@
       <c r="C4">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -463,8 +482,11 @@
       <c r="C5">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -474,8 +496,11 @@
       <c r="C6">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -485,8 +510,11 @@
       <c r="C7">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -496,8 +524,11 @@
       <c r="C8">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -507,8 +538,11 @@
       <c r="C9">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -518,8 +552,11 @@
       <c r="C10">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -529,8 +566,11 @@
       <c r="C11">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -540,8 +580,11 @@
       <c r="C12">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -551,16 +594,22 @@
       <c r="C13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>981348717</v>
       </c>
       <c r="C14">
         <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>